<commit_message>
Filtrando inversores (Em loja) para nova filial Extrema
</commit_message>
<xml_diff>
--- a/calculo_mppt.xlsx
+++ b/calculo_mppt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzo.ferreira\Desktop\dimensionador-fotovoltaico-sigiloso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A0302A-995D-4F30-969A-58985044C99E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18795212-6BC3-4AF3-B352-C54B861FA4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4695" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="421">
   <si>
     <t>Módulo</t>
   </si>
@@ -603,6 +603,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-100KTL-M2 </t>
     </r>
@@ -612,6 +613,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -631,6 +633,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-10K-LCO </t>
     </r>
@@ -640,6 +643,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -665,6 +669,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-15KTL-M5 </t>
     </r>
@@ -674,6 +679,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -699,6 +705,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-20KTL-M5 </t>
     </r>
@@ -708,6 +715,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -727,6 +735,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-250KTL-H1 </t>
     </r>
@@ -736,6 +745,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -755,6 +765,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-25KTL-M5 </t>
     </r>
@@ -764,6 +775,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -789,6 +801,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-3KTL-L1 </t>
     </r>
@@ -798,6 +811,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -832,6 +846,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-5KTL-L1 </t>
     </r>
@@ -841,6 +856,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -866,6 +882,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-6KTL-L1 </t>
     </r>
@@ -875,6 +892,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -906,6 +924,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-75KTL-M1 </t>
     </r>
@@ -915,6 +934,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -934,6 +954,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Huawei SUN2000-8K-LCO </t>
     </r>
@@ -943,6 +964,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>50%</t>
     </r>
@@ -1214,6 +1236,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Solis 75K 5G-PRO </t>
     </r>
@@ -1223,6 +1246,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>com 50%</t>
     </r>
@@ -1239,6 +1263,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Solis S5-GC 37,5K </t>
     </r>
@@ -1248,6 +1273,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>com 50%</t>
     </r>
@@ -1261,6 +1287,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Solis S5-GC 60K </t>
     </r>
@@ -1270,6 +1297,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>com 50%</t>
     </r>
@@ -1316,6 +1344,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Solis-75K-LV-5G-PRO </t>
     </r>
@@ -1325,6 +1354,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>(C/ CONECTOR "Y")</t>
     </r>
@@ -1613,7 +1643,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1622,24 +1652,41 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color indexed="65"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color indexed="2"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1732,21 +1779,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1755,58 +1802,58 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1815,7 +1862,19 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2684,7 +2743,7 @@
       <c r="I3" s="4">
         <v>201741</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="32" t="s">
         <v>62</v>
       </c>
       <c r="L3" s="1" t="s">
@@ -2755,7 +2814,7 @@
       <c r="I4" s="4">
         <v>206291</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="32" t="s">
         <v>62</v>
       </c>
       <c r="L4" s="1" t="s">
@@ -2842,9 +2901,7 @@
       <c r="Q5" s="5">
         <v>167963</v>
       </c>
-      <c r="R5" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R5" s="5"/>
       <c r="S5" s="9">
         <v>40</v>
       </c>
@@ -3051,9 +3108,7 @@
       <c r="Q8" s="8">
         <v>186183</v>
       </c>
-      <c r="R8" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R8" s="8"/>
       <c r="S8" s="6">
         <v>40</v>
       </c>
@@ -3686,9 +3741,7 @@
       <c r="Q17" s="5">
         <v>186177</v>
       </c>
-      <c r="R17" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R17" s="5"/>
       <c r="S17" s="6">
         <v>50</v>
       </c>
@@ -3976,9 +4029,7 @@
       <c r="Q21" s="5">
         <v>167958</v>
       </c>
-      <c r="R21" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R21" s="5"/>
       <c r="S21" s="9">
         <v>35</v>
       </c>
@@ -4054,9 +4105,7 @@
       <c r="Q22" s="8">
         <v>186180</v>
       </c>
-      <c r="R22" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R22" s="8"/>
       <c r="S22" s="6">
         <v>60</v>
       </c>
@@ -5229,8 +5278,12 @@
       <c r="P33" s="1">
         <v>195</v>
       </c>
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
+      <c r="Q33" s="5">
+        <v>90192</v>
+      </c>
+      <c r="R33" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="S33" s="15">
         <v>50</v>
       </c>
@@ -7290,7 +7343,7 @@
         <v>550</v>
       </c>
       <c r="P56" s="1">
-        <v>360</v>
+        <v>90</v>
       </c>
       <c r="Q56" s="5">
         <v>182198</v>
@@ -7422,9 +7475,7 @@
       <c r="Q58" s="11">
         <v>107282</v>
       </c>
-      <c r="R58" s="11" t="s">
-        <v>62</v>
-      </c>
+      <c r="R58" s="11"/>
       <c r="S58" s="9">
         <v>40</v>
       </c>
@@ -7694,9 +7745,7 @@
       <c r="Q60" s="5">
         <v>107277</v>
       </c>
-      <c r="R60" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R60" s="5"/>
       <c r="S60" s="9">
         <v>20</v>
       </c>
@@ -8254,9 +8303,7 @@
       <c r="Q68" s="5">
         <v>107284</v>
       </c>
-      <c r="R68" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R68" s="5"/>
       <c r="S68" s="9">
         <v>115</v>
       </c>
@@ -8581,9 +8628,7 @@
       <c r="Q72" s="5">
         <v>140245</v>
       </c>
-      <c r="R72" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R72" s="5"/>
       <c r="S72" s="9">
         <v>40</v>
       </c>
@@ -8814,9 +8859,7 @@
       <c r="Q75" s="8">
         <v>121772</v>
       </c>
-      <c r="R75" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R75" s="8"/>
       <c r="S75" s="9">
         <v>20</v>
       </c>
@@ -8967,9 +9010,7 @@
       <c r="Q77" s="8">
         <v>140242</v>
       </c>
-      <c r="R77" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R77" s="8"/>
       <c r="S77" s="9">
         <v>40</v>
       </c>
@@ -9431,8 +9472,12 @@
       <c r="P83" s="1">
         <v>50</v>
       </c>
-      <c r="Q83" s="8"/>
-      <c r="R83" s="8"/>
+      <c r="Q83" s="8">
+        <v>170970</v>
+      </c>
+      <c r="R83" s="31" t="s">
+        <v>62</v>
+      </c>
       <c r="S83" s="6">
         <v>20</v>
       </c>
@@ -9617,9 +9662,7 @@
       <c r="Q85" s="8">
         <v>107281</v>
       </c>
-      <c r="R85" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R85" s="8"/>
       <c r="S85" s="9">
         <v>40</v>
       </c>
@@ -10062,9 +10105,7 @@
       <c r="Q89" s="8">
         <v>219935</v>
       </c>
-      <c r="R89" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R89" s="8"/>
       <c r="S89" s="6">
         <v>25</v>
       </c>
@@ -10122,9 +10163,7 @@
       <c r="Q90" s="5">
         <v>219936</v>
       </c>
-      <c r="R90" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R90" s="5"/>
       <c r="S90" s="6">
         <v>24</v>
       </c>
@@ -10188,9 +10227,7 @@
       <c r="Q91" s="8">
         <v>219938</v>
       </c>
-      <c r="R91" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="R91" s="8"/>
       <c r="S91" s="6">
         <v>24</v>
       </c>
@@ -10254,9 +10291,7 @@
       <c r="Q92" s="11">
         <v>219939</v>
       </c>
-      <c r="R92" s="11" t="s">
-        <v>62</v>
-      </c>
+      <c r="R92" s="11"/>
       <c r="S92" s="6">
         <v>24</v>
       </c>
@@ -12019,9 +12054,7 @@
       <c r="Q114" s="5">
         <v>70396</v>
       </c>
-      <c r="R114" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R114" s="5"/>
       <c r="S114" s="15">
         <v>17</v>
       </c>
@@ -12102,9 +12135,7 @@
       <c r="Q115" s="16">
         <v>70397</v>
       </c>
-      <c r="R115" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R115" s="16"/>
       <c r="S115" s="12">
         <v>31.25</v>
       </c>
@@ -12479,9 +12510,7 @@
       <c r="Q122" s="5">
         <v>195100</v>
       </c>
-      <c r="R122" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R122" s="5"/>
       <c r="S122" s="9">
         <v>50</v>
       </c>
@@ -13473,9 +13502,7 @@
       <c r="Q137" s="16">
         <v>215049</v>
       </c>
-      <c r="R137" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R137" s="16"/>
       <c r="S137" s="6">
         <v>40</v>
       </c>
@@ -13516,9 +13543,7 @@
       <c r="Q138" s="5">
         <v>215050</v>
       </c>
-      <c r="R138" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R138" s="5"/>
       <c r="S138" s="6">
         <v>50</v>
       </c>
@@ -13559,9 +13584,7 @@
       <c r="Q139" s="16">
         <v>215051</v>
       </c>
-      <c r="R139" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R139" s="16"/>
       <c r="S139" s="1">
         <v>50</v>
       </c>
@@ -13607,9 +13630,7 @@
       <c r="Q140" s="5">
         <v>215052</v>
       </c>
-      <c r="R140" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R140" s="5"/>
       <c r="S140" s="1">
         <v>50</v>
       </c>
@@ -13649,9 +13670,7 @@
       <c r="Q141" s="16">
         <v>123552</v>
       </c>
-      <c r="R141" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R141" s="16"/>
       <c r="S141" s="1">
         <v>20</v>
       </c>
@@ -13691,9 +13710,7 @@
       <c r="Q142" s="5">
         <v>7490</v>
       </c>
-      <c r="R142" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R142" s="5"/>
       <c r="S142" s="12">
         <v>40</v>
       </c>
@@ -13916,8 +13933,12 @@
       <c r="P144" s="7">
         <v>950</v>
       </c>
-      <c r="Q144" s="5"/>
-      <c r="R144" s="5"/>
+      <c r="Q144" s="5">
+        <v>206226</v>
+      </c>
+      <c r="R144" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="S144" s="1">
         <v>300</v>
       </c>
@@ -14082,9 +14103,7 @@
       <c r="Q147" s="16">
         <v>218759</v>
       </c>
-      <c r="R147" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R147" s="16"/>
       <c r="S147" s="1">
         <v>19.5</v>
       </c>
@@ -14530,9 +14549,7 @@
       <c r="Q153" s="16">
         <v>88619</v>
       </c>
-      <c r="R153" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R153" s="16"/>
       <c r="S153" s="12">
         <v>50</v>
       </c>
@@ -14788,9 +14805,7 @@
       <c r="Q156" s="5">
         <v>75607</v>
       </c>
-      <c r="R156" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R156" s="5"/>
       <c r="S156" s="12">
         <v>40</v>
       </c>
@@ -14948,9 +14963,7 @@
       <c r="Q158" s="5">
         <v>83337</v>
       </c>
-      <c r="R158" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R158" s="5"/>
       <c r="S158" s="12">
         <v>40</v>
       </c>
@@ -15179,8 +15192,12 @@
       <c r="P161" s="7">
         <v>195</v>
       </c>
-      <c r="Q161" s="16"/>
-      <c r="R161" s="16"/>
+      <c r="Q161" s="16">
+        <v>206225</v>
+      </c>
+      <c r="R161" s="30" t="s">
+        <v>62</v>
+      </c>
       <c r="S161" s="1">
         <v>40</v>
       </c>
@@ -15341,9 +15358,7 @@
       <c r="Q164" s="5">
         <v>184846</v>
       </c>
-      <c r="R164" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R164" s="5"/>
       <c r="S164" s="1">
         <v>50</v>
       </c>
@@ -15452,8 +15467,12 @@
       <c r="P165" s="7">
         <v>180</v>
       </c>
-      <c r="Q165" s="16"/>
-      <c r="R165" s="16"/>
+      <c r="Q165" s="16">
+        <v>153075</v>
+      </c>
+      <c r="R165" s="30" t="s">
+        <v>62</v>
+      </c>
       <c r="S165" s="4">
         <v>50</v>
       </c>
@@ -15610,9 +15629,7 @@
       <c r="Q167" s="16">
         <v>105322</v>
       </c>
-      <c r="R167" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R167" s="16"/>
       <c r="S167" s="4">
         <v>22</v>
       </c>
@@ -16259,8 +16276,12 @@
       <c r="P175" s="10">
         <v>180</v>
       </c>
-      <c r="Q175" s="16"/>
-      <c r="R175" s="16"/>
+      <c r="Q175" s="16">
+        <v>152042</v>
+      </c>
+      <c r="R175" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="S175" s="1">
         <v>48</v>
       </c>
@@ -16365,9 +16386,7 @@
       <c r="Q177" s="16">
         <v>152048</v>
       </c>
-      <c r="R177" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R177" s="16"/>
       <c r="S177" s="12">
         <v>60</v>
       </c>
@@ -16429,8 +16448,12 @@
       <c r="P178" s="10">
         <v>180</v>
       </c>
-      <c r="Q178" s="5"/>
-      <c r="R178" s="5"/>
+      <c r="Q178" s="5">
+        <v>152043</v>
+      </c>
+      <c r="R178" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="S178" s="1">
         <v>48</v>
       </c>
@@ -16545,7 +16568,7 @@
         <v>180</v>
       </c>
       <c r="Q180" s="5">
-        <v>52731</v>
+        <v>152045</v>
       </c>
       <c r="R180" s="5" t="s">
         <v>62</v>
@@ -16686,8 +16709,12 @@
       <c r="P182" s="4">
         <v>550</v>
       </c>
-      <c r="Q182" s="5"/>
-      <c r="R182" s="5"/>
+      <c r="Q182" s="5">
+        <v>175388</v>
+      </c>
+      <c r="R182" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="S182" s="6">
         <v>113</v>
       </c>
@@ -16817,8 +16844,12 @@
       <c r="P184" s="4">
         <v>200</v>
       </c>
-      <c r="Q184" s="5"/>
-      <c r="R184" s="5"/>
+      <c r="Q184" s="5">
+        <v>153995</v>
+      </c>
+      <c r="R184" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="S184" s="15">
         <v>48</v>
       </c>
@@ -16963,8 +16994,12 @@
       <c r="P186" s="4">
         <v>250</v>
       </c>
-      <c r="Q186" s="5"/>
-      <c r="R186" s="5"/>
+      <c r="Q186" s="5">
+        <v>160673</v>
+      </c>
+      <c r="R186" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="S186" s="15">
         <v>60</v>
       </c>
@@ -17044,9 +17079,7 @@
       <c r="Q187" s="16">
         <v>152046</v>
       </c>
-      <c r="R187" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R187" s="16"/>
       <c r="S187" s="6">
         <v>48</v>
       </c>
@@ -17519,9 +17552,7 @@
       <c r="Q194" s="5">
         <v>143409</v>
       </c>
-      <c r="R194" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R194" s="5"/>
       <c r="S194" s="15">
         <v>48</v>
       </c>
@@ -17607,9 +17638,7 @@
       <c r="Q195" s="16">
         <v>143408</v>
       </c>
-      <c r="R195" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R195" s="16"/>
       <c r="S195" s="15">
         <v>22.5</v>
       </c>
@@ -17889,9 +17918,7 @@
       <c r="Q199" s="16">
         <v>170120</v>
       </c>
-      <c r="R199" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R199" s="16"/>
       <c r="S199" s="15">
         <v>48</v>
       </c>
@@ -18440,9 +18467,7 @@
       <c r="Q208" s="5">
         <v>143410</v>
       </c>
-      <c r="R208" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R208" s="5"/>
       <c r="S208" s="6">
         <v>60</v>
       </c>
@@ -18519,9 +18544,7 @@
       <c r="Q209" s="16">
         <v>163668</v>
       </c>
-      <c r="R209" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R209" s="16"/>
       <c r="S209" s="15">
         <v>48</v>
       </c>
@@ -18775,9 +18798,7 @@
       <c r="Q212" s="5">
         <v>216764</v>
       </c>
-      <c r="R212" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R212" s="5"/>
       <c r="S212" s="6">
         <v>25</v>
       </c>
@@ -18825,9 +18846,7 @@
       <c r="Q213" s="16">
         <v>216753</v>
       </c>
-      <c r="R213" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R213" s="16"/>
       <c r="S213" s="15">
         <v>40</v>
       </c>
@@ -19070,9 +19089,7 @@
       <c r="Q215" s="16">
         <v>216765</v>
       </c>
-      <c r="R215" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R215" s="16"/>
       <c r="S215" s="6">
         <v>40</v>
       </c>
@@ -19112,9 +19129,7 @@
       <c r="Q216" s="5">
         <v>216766</v>
       </c>
-      <c r="R216" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R216" s="5"/>
       <c r="S216" s="6">
         <v>40</v>
       </c>
@@ -19154,9 +19169,7 @@
       <c r="Q217" s="16">
         <v>216767</v>
       </c>
-      <c r="R217" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R217" s="16"/>
       <c r="S217" s="6">
         <v>40</v>
       </c>
@@ -19326,8 +19339,12 @@
       <c r="P219" s="1">
         <v>250</v>
       </c>
-      <c r="Q219" s="16"/>
-      <c r="R219" s="16"/>
+      <c r="Q219" s="16">
+        <v>206200</v>
+      </c>
+      <c r="R219" s="30" t="s">
+        <v>62</v>
+      </c>
       <c r="S219" s="1">
         <v>40</v>
       </c>
@@ -19373,9 +19390,7 @@
       <c r="Q220" s="5">
         <v>216768</v>
       </c>
-      <c r="R220" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R220" s="5"/>
       <c r="S220" s="1">
         <v>40</v>
       </c>
@@ -19424,9 +19439,7 @@
       <c r="Q221" s="16">
         <v>216769</v>
       </c>
-      <c r="R221" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R221" s="16"/>
       <c r="S221" s="1">
         <v>40</v>
       </c>
@@ -19471,8 +19484,12 @@
       <c r="P222" s="1">
         <v>880</v>
       </c>
-      <c r="Q222" s="5"/>
-      <c r="R222" s="5"/>
+      <c r="Q222" s="5">
+        <v>206199</v>
+      </c>
+      <c r="R222" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="S222" s="12">
         <v>60</v>
       </c>
@@ -19743,9 +19760,7 @@
       <c r="Q224" s="5">
         <v>216770</v>
       </c>
-      <c r="R224" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R224" s="5"/>
       <c r="S224" s="1">
         <v>40</v>
       </c>
@@ -19802,9 +19817,7 @@
       <c r="Q225" s="16">
         <v>216771</v>
       </c>
-      <c r="R225" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R225" s="16"/>
       <c r="S225" s="1">
         <v>40</v>
       </c>
@@ -19862,9 +19875,7 @@
       <c r="Q226" s="5">
         <v>216761</v>
       </c>
-      <c r="R226" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R226" s="5"/>
       <c r="S226" s="1">
         <v>25</v>
       </c>
@@ -19996,9 +20007,7 @@
       <c r="Q228" s="5">
         <v>216762</v>
       </c>
-      <c r="R228" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R228" s="5"/>
       <c r="S228" s="1">
         <v>25</v>
       </c>
@@ -20038,9 +20047,7 @@
       <c r="Q229" s="16">
         <v>216763</v>
       </c>
-      <c r="R229" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R229" s="16"/>
       <c r="S229" s="1">
         <v>25</v>
       </c>
@@ -20088,9 +20095,7 @@
       <c r="Q230" s="5">
         <v>107419</v>
       </c>
-      <c r="R230" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R230" s="5"/>
       <c r="S230" s="15">
         <v>40</v>
       </c>
@@ -20295,9 +20300,7 @@
       <c r="Q232" s="16">
         <v>206201</v>
       </c>
-      <c r="R232" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R232" s="16"/>
       <c r="S232" s="1">
         <v>40</v>
       </c>
@@ -20435,9 +20438,7 @@
       <c r="Q235" s="5">
         <v>206214</v>
       </c>
-      <c r="R235" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="R235" s="5"/>
       <c r="S235" s="1">
         <v>50</v>
       </c>
@@ -20494,9 +20495,7 @@
       <c r="Q236" s="16" t="s">
         <v>420</v>
       </c>
-      <c r="R236" s="16" t="s">
-        <v>62</v>
-      </c>
+      <c r="R236" s="16"/>
       <c r="S236" s="1">
         <v>40</v>
       </c>
@@ -21502,17 +21501,17 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="S88:U88">
     <cfRule type="containsBlanks" dxfId="2" priority="32">
-      <formula>LEN(TRIM(BP88))=0</formula>
+      <formula>LEN(TRIM(BM88))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S3:AG239">
     <cfRule type="containsBlanks" dxfId="1" priority="1">
-      <formula>LEN(TRIM(BP3))=0</formula>
+      <formula>LEN(TRIM(BM3))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH3:AV239">
     <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(CE3))=0</formula>
+      <formula>LEN(TRIM(CB3))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0" footer="0"/>

</xml_diff>

<commit_message>
Adicionando Sungrow para filial Extrema
</commit_message>
<xml_diff>
--- a/calculo_mppt.xlsx
+++ b/calculo_mppt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzo.ferreira\Desktop\dimensionador-fotovoltaico-sigiloso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18795212-6BC3-4AF3-B352-C54B861FA4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0225D6-CB2A-4CC3-A05B-F9656C52F5A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4695" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="421">
   <si>
     <t>Módulo</t>
   </si>
@@ -1779,7 +1779,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1875,6 +1875,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -18798,7 +18801,9 @@
       <c r="Q212" s="5">
         <v>216764</v>
       </c>
-      <c r="R212" s="5"/>
+      <c r="R212" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="S212" s="6">
         <v>25</v>
       </c>
@@ -19089,7 +19094,9 @@
       <c r="Q215" s="16">
         <v>216765</v>
       </c>
-      <c r="R215" s="16"/>
+      <c r="R215" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="S215" s="6">
         <v>40</v>
       </c>
@@ -19129,7 +19136,9 @@
       <c r="Q216" s="5">
         <v>216766</v>
       </c>
-      <c r="R216" s="5"/>
+      <c r="R216" s="33" t="s">
+        <v>62</v>
+      </c>
       <c r="S216" s="6">
         <v>40</v>
       </c>
@@ -20007,7 +20016,9 @@
       <c r="Q228" s="5">
         <v>216762</v>
       </c>
-      <c r="R228" s="5"/>
+      <c r="R228" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="S228" s="1">
         <v>25</v>
       </c>
@@ -20047,7 +20058,9 @@
       <c r="Q229" s="16">
         <v>216763</v>
       </c>
-      <c r="R229" s="16"/>
+      <c r="R229" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="S229" s="1">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
adição novos inversores huawei filial extrema
</commit_message>
<xml_diff>
--- a/calculo_mppt.xlsx
+++ b/calculo_mppt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\enzo.ferreira\Desktop\dimensionador-fotovoltaico-sigiloso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C5C96A-C3BB-4906-B78A-A85C5553D34A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7769FE1B-8307-45D7-97EE-5DF5B80A2036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4695" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="422">
   <si>
     <t>Módulo</t>
   </si>
@@ -1637,6 +1637,9 @@
   </si>
   <si>
     <t xml:space="preserve">206195	</t>
+  </si>
+  <si>
+    <t>HUAWEI 50KW T220 ON (50K-MGL0-BR)</t>
   </si>
 </sst>
 </file>
@@ -7745,7 +7748,9 @@
       <c r="Q60" s="5">
         <v>107277</v>
       </c>
-      <c r="R60" s="5"/>
+      <c r="R60" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="S60" s="9">
         <v>20</v>
       </c>
@@ -8859,7 +8864,9 @@
       <c r="Q75" s="8">
         <v>121772</v>
       </c>
-      <c r="R75" s="8"/>
+      <c r="R75" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="S75" s="9">
         <v>20</v>
       </c>
@@ -20626,8 +20633,90 @@
       </c>
     </row>
     <row r="237" spans="12:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="Q237" s="5"/>
-      <c r="R237" s="5"/>
+      <c r="L237" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="M237" s="1">
+        <v>50</v>
+      </c>
+      <c r="N237" s="1">
+        <v>100000</v>
+      </c>
+      <c r="O237" s="1">
+        <v>750</v>
+      </c>
+      <c r="P237" s="1">
+        <v>160</v>
+      </c>
+      <c r="Q237" s="5">
+        <v>183058</v>
+      </c>
+      <c r="R237" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="S237" s="1">
+        <v>66</v>
+      </c>
+      <c r="T237" s="1">
+        <v>66</v>
+      </c>
+      <c r="U237" s="1">
+        <v>66</v>
+      </c>
+      <c r="V237" s="1">
+        <v>66</v>
+      </c>
+      <c r="W237" s="1">
+        <v>66</v>
+      </c>
+      <c r="X237" s="1">
+        <v>66</v>
+      </c>
+      <c r="Y237" s="1">
+        <v>66</v>
+      </c>
+      <c r="AH237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AI237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AJ237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AK237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AL237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AM237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AN237" s="1">
+        <v>48</v>
+      </c>
+      <c r="AW237" s="1">
+        <v>3</v>
+      </c>
+      <c r="AX237" s="1">
+        <v>3</v>
+      </c>
+      <c r="AY237" s="1">
+        <v>3</v>
+      </c>
+      <c r="AZ237" s="1">
+        <v>3</v>
+      </c>
+      <c r="BA237" s="1">
+        <v>3</v>
+      </c>
+      <c r="BB237" s="1">
+        <v>3</v>
+      </c>
+      <c r="BC237" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="238" spans="12:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="Q238" s="16"/>

</xml_diff>